<commit_message>
Work Plan (5th Month)
</commit_message>
<xml_diff>
--- a/5th month plan.xlsx
+++ b/5th month plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Daily-GitHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED6C748F-5BC6-433E-B747-2A61E5D10546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3826D3EF-696F-44A0-8E48-D72EE8FA6697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7FFA0864-4158-47B6-89E4-68EED148B573}"/>
+    <workbookView xWindow="4152" yWindow="2112" windowWidth="17280" windowHeight="9960" xr2:uid="{7FFA0864-4158-47B6-89E4-68EED148B573}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="85">
   <si>
     <t>Concept Focus</t>
   </si>
@@ -282,7 +282,13 @@
     <t>Stacks, Queue Simulation</t>
   </si>
   <si>
-    <t>Review &amp; Wrap-up Month 5</t>
+    <t>Arrays - DS</t>
+  </si>
+  <si>
+    <t>https://www.hackerrank.com/challenges/arrays-ds/problem</t>
+  </si>
+  <si>
+    <t>Reverse Vector</t>
   </si>
 </sst>
 </file>
@@ -1180,21 +1186,21 @@
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>150</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>2</v>
+        <v>82</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1219,6 +1225,7 @@
     <hyperlink ref="D27" r:id="rId18" xr:uid="{360B69C2-8981-470A-BBC0-4A6B52F7E260}"/>
     <hyperlink ref="D28" r:id="rId19" xr:uid="{86DD4016-A526-49B1-BC0E-957AC2CDFE2A}"/>
     <hyperlink ref="D30" r:id="rId20" xr:uid="{6AEA9D87-C90C-470F-8E1B-3FB50B06B8F6}"/>
+    <hyperlink ref="D31" r:id="rId21" xr:uid="{0843BE40-6F42-470B-A698-CB40D785139C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>